<commit_message>
Give a record member's elements one discriminator, not one each
The fixture grows the three record shapes with a member that reaches
several tables: an array of records, a record of one, and a record whose
members are the arrays. All three convert already - the member carries
the key, narrowed to the target's type - and none of them get accessors,
which is what this branch is for.

The first thing that showed is the naming. An array of two elements is a
column per element, and the discriminator was named after the column, so
one member declared `LoadoutSlot1PickTarget` and
`LoadoutSlot2PickTarget` for the same question. It is named after the
member now - group plus the path that reaches the leaf, because a leaf
does not carry its own path and the last part alone would collide
between levels - and every element of that member points at the one
type.

The declaration itself moved into a helper so the member walk and the
plain-column walk cannot drift apart.
</commit_message>
<xml_diff>
--- a/test/fixtures/xlsx/multi-target/multi-target.xlsx
+++ b/test/fixtures/xlsx/multi-target/multi-target.xlsx
@@ -8,12 +8,13 @@
   <sheets>
     <sheet name="Catalogues" sheetId="1" r:id="rId3"/>
     <sheet name="Holders" sheetId="2" r:id="rId4"/>
+    <sheet name="Groups" sheetId="3" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="93">
   <si>
     <t xml:space="preserve">~~table:Weapon~~</t>
   </si>
@@ -196,6 +197,102 @@
   </si>
   <si>
     <t xml:space="preserve">3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~~table:Loadout~~</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A record array whose member reaches several tables.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slot1.Pick</t>
+  </si>
+  <si>
+    <t xml:space="preserve">element 1 - two targets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slot1.Count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">element 1 - an ordinary member</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slot2.Pick</t>
+  </si>
+  <si>
+    <t xml:space="preserve">element 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slot2.Count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~~table:Fitting~~</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One record - no element number at all - whose member reaches several.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Main.Pick</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the member, in a record of one</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Main.Count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">an ordinary member beside it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">padding, so every table is one width</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pad2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~~table:Rack~~</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One record whose members are arrays, one of them reaching several.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slots.Pick1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">element 1 of the member</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slots.Pick2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">element 2 of the member</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slots.Count1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">element 1 beside it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slots.Count2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">element 2 beside it</t>
   </si>
 </sst>
 </file>
@@ -765,4 +862,365 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="B2:V10"/>
+  <sheetFormatPr defaultColWidth="8.43" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="2">
+      <c r="B2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J2" t="s">
+        <v>71</v>
+      </c>
+      <c r="R2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="s">
+        <v>62</v>
+      </c>
+      <c r="J3" t="s">
+        <v>72</v>
+      </c>
+      <c r="R3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E4" t="s">
+        <v>67</v>
+      </c>
+      <c r="F4" t="s">
+        <v>69</v>
+      </c>
+      <c r="J4" t="s">
+        <v>2</v>
+      </c>
+      <c r="K4" t="s">
+        <v>73</v>
+      </c>
+      <c r="L4" t="s">
+        <v>75</v>
+      </c>
+      <c r="M4" t="s">
+        <v>77</v>
+      </c>
+      <c r="N4" t="s">
+        <v>79</v>
+      </c>
+      <c r="R4" t="s">
+        <v>2</v>
+      </c>
+      <c r="S4" t="s">
+        <v>85</v>
+      </c>
+      <c r="T4" t="s">
+        <v>87</v>
+      </c>
+      <c r="U4" t="s">
+        <v>89</v>
+      </c>
+      <c r="V4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D5" t="s">
+        <v>66</v>
+      </c>
+      <c r="E5" t="s">
+        <v>68</v>
+      </c>
+      <c r="F5" t="s">
+        <v>68</v>
+      </c>
+      <c r="J5" t="s">
+        <v>43</v>
+      </c>
+      <c r="K5" t="s">
+        <v>74</v>
+      </c>
+      <c r="L5" t="s">
+        <v>76</v>
+      </c>
+      <c r="M5" t="s">
+        <v>78</v>
+      </c>
+      <c r="N5" t="s">
+        <v>78</v>
+      </c>
+      <c r="R5" t="s">
+        <v>43</v>
+      </c>
+      <c r="S5" t="s">
+        <v>86</v>
+      </c>
+      <c r="T5" t="s">
+        <v>88</v>
+      </c>
+      <c r="U5" t="s">
+        <v>90</v>
+      </c>
+      <c r="V5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" t="s">
+        <v>4</v>
+      </c>
+      <c r="E6" t="s">
+        <v>46</v>
+      </c>
+      <c r="F6" t="s">
+        <v>4</v>
+      </c>
+      <c r="J6" t="s">
+        <v>4</v>
+      </c>
+      <c r="K6" t="s">
+        <v>46</v>
+      </c>
+      <c r="L6" t="s">
+        <v>4</v>
+      </c>
+      <c r="M6" t="s">
+        <v>4</v>
+      </c>
+      <c r="N6" t="s">
+        <v>4</v>
+      </c>
+      <c r="R6" t="s">
+        <v>4</v>
+      </c>
+      <c r="S6" t="s">
+        <v>46</v>
+      </c>
+      <c r="T6" t="s">
+        <v>46</v>
+      </c>
+      <c r="U6" t="s">
+        <v>4</v>
+      </c>
+      <c r="V6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7" t="s">
+        <v>5</v>
+      </c>
+      <c r="E7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F7" t="s">
+        <v>5</v>
+      </c>
+      <c r="J7" t="s">
+        <v>5</v>
+      </c>
+      <c r="K7" t="s">
+        <v>47</v>
+      </c>
+      <c r="L7" t="s">
+        <v>5</v>
+      </c>
+      <c r="M7" t="s">
+        <v>5</v>
+      </c>
+      <c r="N7" t="s">
+        <v>5</v>
+      </c>
+      <c r="R7" t="s">
+        <v>5</v>
+      </c>
+      <c r="S7" t="s">
+        <v>47</v>
+      </c>
+      <c r="T7" t="s">
+        <v>47</v>
+      </c>
+      <c r="U7" t="s">
+        <v>5</v>
+      </c>
+      <c r="V7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" t="s">
+        <v>6</v>
+      </c>
+      <c r="F8" t="s">
+        <v>6</v>
+      </c>
+      <c r="J8" t="s">
+        <v>6</v>
+      </c>
+      <c r="K8" t="s">
+        <v>6</v>
+      </c>
+      <c r="L8" t="s">
+        <v>6</v>
+      </c>
+      <c r="M8" t="s">
+        <v>6</v>
+      </c>
+      <c r="N8" t="s">
+        <v>6</v>
+      </c>
+      <c r="R8" t="s">
+        <v>6</v>
+      </c>
+      <c r="S8" t="s">
+        <v>6</v>
+      </c>
+      <c r="T8" t="s">
+        <v>6</v>
+      </c>
+      <c r="U8" t="s">
+        <v>6</v>
+      </c>
+      <c r="V8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" t="s">
+        <v>57</v>
+      </c>
+      <c r="E9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9" t="s">
+        <v>58</v>
+      </c>
+      <c r="J9" t="s">
+        <v>57</v>
+      </c>
+      <c r="K9" t="s">
+        <v>20</v>
+      </c>
+      <c r="L9" t="s">
+        <v>80</v>
+      </c>
+      <c r="M9" t="s">
+        <v>81</v>
+      </c>
+      <c r="N9" t="s">
+        <v>81</v>
+      </c>
+      <c r="R9" t="s">
+        <v>57</v>
+      </c>
+      <c r="S9" t="s">
+        <v>12</v>
+      </c>
+      <c r="T9" t="s">
+        <v>22</v>
+      </c>
+      <c r="U9" t="s">
+        <v>12</v>
+      </c>
+      <c r="V9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" t="s">
+        <v>60</v>
+      </c>
+      <c r="E10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" t="s">
+        <v>70</v>
+      </c>
+      <c r="J10" t="s">
+        <v>58</v>
+      </c>
+      <c r="K10" t="s">
+        <v>15</v>
+      </c>
+      <c r="L10" t="s">
+        <v>82</v>
+      </c>
+      <c r="M10" t="s">
+        <v>81</v>
+      </c>
+      <c r="N10" t="s">
+        <v>81</v>
+      </c>
+      <c r="R10" t="s">
+        <v>58</v>
+      </c>
+      <c r="S10" t="s">
+        <v>20</v>
+      </c>
+      <c r="T10" t="s">
+        <v>15</v>
+      </c>
+      <c r="U10" t="s">
+        <v>26</v>
+      </c>
+      <c r="V10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>